<commit_message>
Add sales-based depletion forecast for storage until November
Прогноз хранения до 01.11 с учётом текущего темпа продаж: остаток
списывается ежедневно, хранение начисляется на остаток до распродажи.
Итог с продажами: 605 097 руб против 814 657 руб без продаж.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RrW5WcYKgjMut1vasTMe2Q
</commit_message>
<xml_diff>
--- a/outputs/Хранение_до_ноября_без_ЧЗ.xlsx
+++ b/outputs/Хранение_до_ноября_без_ЧЗ.xlsx
@@ -40,7 +40,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -55,6 +55,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -84,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -96,6 +101,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -462,15 +468,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="62" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,12 +504,22 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Хранение до ноября за ед. (129 дн), руб</t>
+          <t>Хранение до ноября всего (без продаж), руб</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Хранение до ноября всего, руб</t>
+          <t>Продажи в день, шт (тек. темп)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Прогноз остатка к 01.11, шт</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Хранение до ноября с учётом продаж, руб</t>
         </is>
       </c>
     </row>
@@ -521,10 +539,16 @@
         <v>0.1612</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>20.79</v>
+        <v>11561.91</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>11561.91</v>
+        <v>1</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>427</v>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>10231.04</v>
       </c>
     </row>
     <row r="3">
@@ -543,10 +567,16 @@
         <v>0.1595</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>20.58</v>
+        <v>1502.01</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>1502.01</v>
+        <v>0.12</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>1337.41</v>
       </c>
     </row>
     <row r="4">
@@ -565,10 +595,16 @@
         <v>0.4148</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>53.51</v>
+        <v>6688.65</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>6688.65</v>
+        <v>1.25</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>2618.43</v>
       </c>
     </row>
     <row r="5">
@@ -587,10 +623,16 @@
         <v>0.2808</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>36.22</v>
+        <v>5216.14</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>5216.14</v>
+        <v>0.75</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>3477.43</v>
       </c>
     </row>
     <row r="6">
@@ -609,10 +651,16 @@
         <v>0.1588</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>20.49</v>
+        <v>11266.86</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>11266.86</v>
+        <v>1.38</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>373</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>9464.16</v>
       </c>
     </row>
     <row r="7">
@@ -631,10 +679,16 @@
         <v>0.9546</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>123.14</v>
+        <v>75117.47</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>75117.47</v>
+        <v>2.88</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>239</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>52459.09</v>
       </c>
     </row>
     <row r="8">
@@ -653,10 +707,16 @@
         <v>0.1485</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>19.16</v>
+        <v>3563.11</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>3563.11</v>
+        <v>2.38</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>1095.43</v>
       </c>
     </row>
     <row r="9">
@@ -675,10 +735,16 @@
         <v>0.1653</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>21.32</v>
+        <v>2132.37</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>2132.37</v>
+        <v>7</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>126.45</v>
       </c>
     </row>
     <row r="10">
@@ -697,10 +763,16 @@
         <v>0.1643</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>21.19</v>
+        <v>10512.57</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>10512.57</v>
+        <v>0.5</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>432</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>9834.34</v>
       </c>
     </row>
     <row r="11">
@@ -719,10 +791,16 @@
         <v>0.1704</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>21.98</v>
+        <v>3956.69</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>3956.69</v>
+        <v>3.62</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>776.92</v>
       </c>
     </row>
     <row r="12">
@@ -741,9 +819,15 @@
         <v>0.148</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>19.09</v>
+        <v>954.6</v>
       </c>
       <c r="F12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="H12" s="5" t="n">
         <v>954.6</v>
       </c>
     </row>
@@ -763,9 +847,15 @@
         <v>0.1647</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>21.25</v>
+        <v>7329.97</v>
       </c>
       <c r="F13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>345</v>
+      </c>
+      <c r="H13" s="5" t="n">
         <v>7329.97</v>
       </c>
     </row>
@@ -785,10 +875,16 @@
         <v>0.1545</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>19.93</v>
+        <v>22082.99</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>22082.99</v>
+        <v>4</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>592</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>16980.79</v>
       </c>
     </row>
     <row r="15">
@@ -807,10 +903,16 @@
         <v>0.1355</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>17.48</v>
+        <v>43960.94</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>43960.94</v>
+        <v>23.75</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>18214.08</v>
       </c>
     </row>
     <row r="16">
@@ -829,10 +931,16 @@
         <v>0.135</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>17.42</v>
+        <v>48013.16</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>48013.16</v>
+        <v>4.62</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>2160</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>42858.31</v>
       </c>
     </row>
     <row r="17">
@@ -851,9 +959,15 @@
         <v>0.1419</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>18.31</v>
+        <v>0</v>
       </c>
       <c r="F17" s="5" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -873,10 +987,16 @@
         <v>0.1216</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>15.69</v>
+        <v>8015.75</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>8015.75</v>
+        <v>3.38</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>76</v>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>4627.49</v>
       </c>
     </row>
     <row r="19">
@@ -895,10 +1015,16 @@
         <v>0.1506</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>19.43</v>
+        <v>1670.76</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>1670.76</v>
+        <v>1.5</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>377.78</v>
       </c>
     </row>
     <row r="20">
@@ -917,10 +1043,16 @@
         <v>0.1623</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>20.94</v>
+        <v>29541.68</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>29541.68</v>
+        <v>4.12</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>879</v>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>24014.39</v>
       </c>
     </row>
     <row r="21">
@@ -939,10 +1071,16 @@
         <v>0.1359</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>17.53</v>
+        <v>10115.44</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>10115.44</v>
+        <v>9.619999999999999</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>2389.63</v>
       </c>
     </row>
     <row r="22">
@@ -961,10 +1099,16 @@
         <v>0.1526</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>19.69</v>
+        <v>4626.07</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>4626.07</v>
+        <v>5</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>860.66</v>
       </c>
     </row>
     <row r="23">
@@ -983,10 +1127,16 @@
         <v>0.1653</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>21.32</v>
+        <v>639.71</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>639.71</v>
+        <v>4.5</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>19.09</v>
       </c>
     </row>
     <row r="24">
@@ -1005,10 +1155,16 @@
         <v>0.1504</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>19.4</v>
+        <v>15404.87</v>
       </c>
       <c r="F24" s="5" t="n">
-        <v>15404.87</v>
+        <v>4.12</v>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>262</v>
+      </c>
+      <c r="H24" s="5" t="n">
+        <v>10282.85</v>
       </c>
     </row>
     <row r="25">
@@ -1027,10 +1183,16 @@
         <v>0.1492</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>19.25</v>
+        <v>16629.24</v>
       </c>
       <c r="F25" s="5" t="n">
-        <v>16629.24</v>
+        <v>2.25</v>
+      </c>
+      <c r="G25" s="3" t="n">
+        <v>574</v>
+      </c>
+      <c r="H25" s="5" t="n">
+        <v>13857.7</v>
       </c>
     </row>
     <row r="26">
@@ -1049,10 +1211,16 @@
         <v>0.1514</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>19.53</v>
+        <v>18261.11</v>
       </c>
       <c r="F26" s="5" t="n">
-        <v>18261.11</v>
+        <v>1</v>
+      </c>
+      <c r="G26" s="3" t="n">
+        <v>806</v>
+      </c>
+      <c r="H26" s="5" t="n">
+        <v>17011.15</v>
       </c>
     </row>
     <row r="27">
@@ -1071,10 +1239,16 @@
         <v>0.1633</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>21.07</v>
+        <v>7857.51</v>
       </c>
       <c r="F27" s="5" t="n">
-        <v>7857.51</v>
+        <v>13.12</v>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="5" t="n">
+        <v>896.23</v>
       </c>
     </row>
     <row r="28">
@@ -1093,10 +1267,16 @@
         <v>0.0925</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>11.93</v>
+        <v>8651.059999999999</v>
       </c>
       <c r="F28" s="5" t="n">
-        <v>8651.059999999999</v>
+        <v>2</v>
+      </c>
+      <c r="G28" s="3" t="n">
+        <v>467</v>
+      </c>
+      <c r="H28" s="5" t="n">
+        <v>7123.7</v>
       </c>
     </row>
     <row r="29">
@@ -1115,10 +1295,16 @@
         <v>0.1858</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>23.97</v>
+        <v>6327.6</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>6327.6</v>
+        <v>2.12</v>
+      </c>
+      <c r="G29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="5" t="n">
+        <v>3071.51</v>
       </c>
     </row>
     <row r="30">
@@ -1137,10 +1323,16 @@
         <v>0.3027</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>39.05</v>
+        <v>127609.84</v>
       </c>
       <c r="F30" s="5" t="n">
-        <v>127609.84</v>
+        <v>14.38</v>
+      </c>
+      <c r="G30" s="3" t="n">
+        <v>1414</v>
+      </c>
+      <c r="H30" s="5" t="n">
+        <v>91685.41</v>
       </c>
     </row>
     <row r="31">
@@ -1159,10 +1351,16 @@
         <v>0.2001</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>25.81</v>
+        <v>107923.73</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>107923.73</v>
+        <v>9.880000000000001</v>
+      </c>
+      <c r="G31" s="3" t="n">
+        <v>2907</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>91609.98</v>
       </c>
     </row>
     <row r="32">
@@ -1181,10 +1379,16 @@
         <v>0.1512</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>19.5</v>
+        <v>11605.36</v>
       </c>
       <c r="F32" s="5" t="n">
-        <v>11605.36</v>
+        <v>5.5</v>
+      </c>
+      <c r="G32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="5" t="n">
+        <v>4911.28</v>
       </c>
     </row>
     <row r="33">
@@ -1203,10 +1407,16 @@
         <v>0.1447</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>18.67</v>
+        <v>9613.139999999999</v>
       </c>
       <c r="F33" s="5" t="n">
-        <v>9613.139999999999</v>
+        <v>1.12</v>
+      </c>
+      <c r="G33" s="3" t="n">
+        <v>370</v>
+      </c>
+      <c r="H33" s="5" t="n">
+        <v>8269.17</v>
       </c>
     </row>
     <row r="34">
@@ -1225,10 +1435,16 @@
         <v>0.1519</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>19.6</v>
+        <v>2135.87</v>
       </c>
       <c r="F34" s="5" t="n">
-        <v>2135.87</v>
+        <v>1.5</v>
+      </c>
+      <c r="G34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="5" t="n">
+        <v>609.88</v>
       </c>
     </row>
     <row r="35">
@@ -1247,10 +1463,16 @@
         <v>0.1359</v>
       </c>
       <c r="E35" s="5" t="n">
-        <v>17.53</v>
+        <v>753.84</v>
       </c>
       <c r="F35" s="5" t="n">
-        <v>753.84</v>
+        <v>0.25</v>
+      </c>
+      <c r="G35" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="H35" s="5" t="n">
+        <v>473.34</v>
       </c>
     </row>
     <row r="36">
@@ -1269,10 +1491,16 @@
         <v>0.1612</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>20.79</v>
+        <v>2661.73</v>
       </c>
       <c r="F36" s="5" t="n">
-        <v>2661.73</v>
+        <v>1</v>
+      </c>
+      <c r="G36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="5" t="n">
+        <v>1330.87</v>
       </c>
     </row>
     <row r="37">
@@ -1291,10 +1519,16 @@
         <v>0.1834</v>
       </c>
       <c r="E37" s="5" t="n">
-        <v>23.66</v>
+        <v>32719.84</v>
       </c>
       <c r="F37" s="5" t="n">
-        <v>32719.84</v>
+        <v>0.88</v>
+      </c>
+      <c r="G37" s="3" t="n">
+        <v>1270</v>
+      </c>
+      <c r="H37" s="5" t="n">
+        <v>31394.96</v>
       </c>
     </row>
     <row r="38">
@@ -1313,10 +1547,16 @@
         <v>0.1891</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>24.39</v>
+        <v>25418.44</v>
       </c>
       <c r="F38" s="5" t="n">
-        <v>25418.44</v>
+        <v>1.62</v>
+      </c>
+      <c r="G38" s="3" t="n">
+        <v>832</v>
+      </c>
+      <c r="H38" s="5" t="n">
+        <v>22881.48</v>
       </c>
     </row>
     <row r="39">
@@ -1335,10 +1575,16 @@
         <v>0.1844</v>
       </c>
       <c r="E39" s="5" t="n">
-        <v>23.79</v>
+        <v>19862.65</v>
       </c>
       <c r="F39" s="5" t="n">
-        <v>19862.65</v>
+        <v>1.75</v>
+      </c>
+      <c r="G39" s="3" t="n">
+        <v>609</v>
+      </c>
+      <c r="H39" s="5" t="n">
+        <v>17198.43</v>
       </c>
     </row>
     <row r="40">
@@ -1357,10 +1603,16 @@
         <v>0.1534</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>19.79</v>
+        <v>8311.209999999999</v>
       </c>
       <c r="F40" s="5" t="n">
-        <v>8311.209999999999</v>
+        <v>0.12</v>
+      </c>
+      <c r="G40" s="3" t="n">
+        <v>404</v>
+      </c>
+      <c r="H40" s="5" t="n">
+        <v>8152.9</v>
       </c>
     </row>
     <row r="41">
@@ -1379,10 +1631,16 @@
         <v>0.1502</v>
       </c>
       <c r="E41" s="5" t="n">
-        <v>19.38</v>
+        <v>12284.26</v>
       </c>
       <c r="F41" s="5" t="n">
-        <v>12284.26</v>
+        <v>6.75</v>
+      </c>
+      <c r="G41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="5" t="n">
+        <v>4519.78</v>
       </c>
     </row>
     <row r="42">
@@ -1401,10 +1659,16 @@
         <v>0.3346</v>
       </c>
       <c r="E42" s="5" t="n">
-        <v>43.16</v>
+        <v>5136.44</v>
       </c>
       <c r="F42" s="5" t="n">
-        <v>5136.44</v>
+        <v>0.25</v>
+      </c>
+      <c r="G42" s="3" t="n">
+        <v>87</v>
+      </c>
+      <c r="H42" s="5" t="n">
+        <v>4445.83</v>
       </c>
     </row>
     <row r="43">
@@ -1423,10 +1687,16 @@
         <v>0.1333</v>
       </c>
       <c r="E43" s="5" t="n">
-        <v>17.2</v>
+        <v>1805.55</v>
       </c>
       <c r="F43" s="5" t="n">
-        <v>1805.55</v>
+        <v>0.88</v>
+      </c>
+      <c r="G43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="5" t="n">
+        <v>846.79</v>
       </c>
     </row>
     <row r="44">
@@ -1445,10 +1715,16 @@
         <v>0.1553</v>
       </c>
       <c r="E44" s="5" t="n">
-        <v>20.03</v>
+        <v>6010.11</v>
       </c>
       <c r="F44" s="5" t="n">
-        <v>6010.11</v>
+        <v>1.25</v>
+      </c>
+      <c r="G44" s="3" t="n">
+        <v>139</v>
+      </c>
+      <c r="H44" s="5" t="n">
+        <v>4407.41</v>
       </c>
     </row>
     <row r="45">
@@ -1467,10 +1743,16 @@
         <v>0.1301</v>
       </c>
       <c r="E45" s="5" t="n">
-        <v>16.78</v>
+        <v>4531.38</v>
       </c>
       <c r="F45" s="5" t="n">
-        <v>4531.38</v>
+        <v>0.5</v>
+      </c>
+      <c r="G45" s="3" t="n">
+        <v>206</v>
+      </c>
+      <c r="H45" s="5" t="n">
+        <v>3994.33</v>
       </c>
     </row>
     <row r="46">
@@ -1489,10 +1771,16 @@
         <v>0.1535</v>
       </c>
       <c r="E46" s="5" t="n">
-        <v>19.8</v>
+        <v>11029.44</v>
       </c>
       <c r="F46" s="5" t="n">
-        <v>11029.44</v>
+        <v>1.38</v>
+      </c>
+      <c r="G46" s="3" t="n">
+        <v>380</v>
+      </c>
+      <c r="H46" s="5" t="n">
+        <v>9286.9</v>
       </c>
     </row>
     <row r="47">
@@ -1511,10 +1799,16 @@
         <v>0.1651</v>
       </c>
       <c r="E47" s="5" t="n">
-        <v>21.3</v>
+        <v>4472.56</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>4472.56</v>
+        <v>1.75</v>
+      </c>
+      <c r="G47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="5" t="n">
+        <v>2097.6</v>
       </c>
     </row>
     <row r="48">
@@ -1533,10 +1827,16 @@
         <v>0.1584</v>
       </c>
       <c r="E48" s="5" t="n">
-        <v>20.43</v>
+        <v>1532.52</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>1532.52</v>
+        <v>1</v>
+      </c>
+      <c r="G48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="5" t="n">
+        <v>451.44</v>
       </c>
     </row>
     <row r="49">
@@ -1555,10 +1855,16 @@
         <v>0.148</v>
       </c>
       <c r="E49" s="5" t="n">
-        <v>19.09</v>
+        <v>1699.19</v>
       </c>
       <c r="F49" s="5" t="n">
-        <v>1699.19</v>
+        <v>0.25</v>
+      </c>
+      <c r="G49" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="H49" s="5" t="n">
+        <v>1393.72</v>
       </c>
     </row>
     <row r="50">
@@ -1577,10 +1883,16 @@
         <v>0.1449</v>
       </c>
       <c r="E50" s="5" t="n">
-        <v>18.69</v>
+        <v>1551.44</v>
       </c>
       <c r="F50" s="5" t="n">
-        <v>1551.44</v>
+        <v>0.25</v>
+      </c>
+      <c r="G50" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="H50" s="5" t="n">
+        <v>1252.37</v>
       </c>
     </row>
     <row r="51">
@@ -1599,10 +1911,16 @@
         <v>0.1381</v>
       </c>
       <c r="E51" s="5" t="n">
-        <v>17.81</v>
+        <v>9388.450000000001</v>
       </c>
       <c r="F51" s="5" t="n">
-        <v>9388.450000000001</v>
+        <v>0.12</v>
+      </c>
+      <c r="G51" s="3" t="n">
+        <v>511</v>
+      </c>
+      <c r="H51" s="5" t="n">
+        <v>9245.93</v>
       </c>
     </row>
     <row r="52">
@@ -1621,10 +1939,16 @@
         <v>0.1671</v>
       </c>
       <c r="E52" s="5" t="n">
-        <v>21.56</v>
+        <v>1185.57</v>
       </c>
       <c r="F52" s="5" t="n">
-        <v>1185.57</v>
+        <v>0.25</v>
+      </c>
+      <c r="G52" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="H52" s="5" t="n">
+        <v>840.6799999999999</v>
       </c>
     </row>
     <row r="53">
@@ -1643,10 +1967,16 @@
         <v>0.16</v>
       </c>
       <c r="E53" s="5" t="n">
-        <v>20.64</v>
+        <v>2435.52</v>
       </c>
       <c r="F53" s="5" t="n">
-        <v>2435.52</v>
+        <v>0.75</v>
+      </c>
+      <c r="G53" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="H53" s="5" t="n">
+        <v>1444.8</v>
       </c>
     </row>
     <row r="54">
@@ -1665,10 +1995,16 @@
         <v>0.154</v>
       </c>
       <c r="E54" s="5" t="n">
-        <v>19.87</v>
+        <v>635.71</v>
       </c>
       <c r="F54" s="5" t="n">
-        <v>635.71</v>
+        <v>0.12</v>
+      </c>
+      <c r="G54" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="H54" s="5" t="n">
+        <v>476.78</v>
       </c>
     </row>
     <row r="55">
@@ -1687,10 +2023,16 @@
         <v>0.1588</v>
       </c>
       <c r="E55" s="5" t="n">
-        <v>20.49</v>
+        <v>2028.03</v>
       </c>
       <c r="F55" s="5" t="n">
-        <v>2028.03</v>
+        <v>0.12</v>
+      </c>
+      <c r="G55" s="3" t="n">
+        <v>83</v>
+      </c>
+      <c r="H55" s="5" t="n">
+        <v>1864.15</v>
       </c>
     </row>
     <row r="56">
@@ -1709,10 +2051,16 @@
         <v>0.1647</v>
       </c>
       <c r="E56" s="5" t="n">
-        <v>21.25</v>
+        <v>10644.4</v>
       </c>
       <c r="F56" s="5" t="n">
-        <v>10644.4</v>
+        <v>0.25</v>
+      </c>
+      <c r="G56" s="3" t="n">
+        <v>469</v>
+      </c>
+      <c r="H56" s="5" t="n">
+        <v>10304.46</v>
       </c>
     </row>
     <row r="57">
@@ -1731,10 +2079,16 @@
         <v>0.1587</v>
       </c>
       <c r="E57" s="5" t="n">
-        <v>20.47</v>
+        <v>1719.67</v>
       </c>
       <c r="F57" s="5" t="n">
-        <v>1719.67</v>
+        <v>0.5</v>
+      </c>
+      <c r="G57" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H57" s="5" t="n">
+        <v>1064.56</v>
       </c>
     </row>
     <row r="58">
@@ -1753,9 +2107,15 @@
         <v>0.1619</v>
       </c>
       <c r="E58" s="5" t="n">
-        <v>20.89</v>
+        <v>2589.75</v>
       </c>
       <c r="F58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" s="3" t="n">
+        <v>124</v>
+      </c>
+      <c r="H58" s="5" t="n">
         <v>2589.75</v>
       </c>
     </row>
@@ -1775,9 +2135,15 @@
         <v>0.1503</v>
       </c>
       <c r="E59" s="5" t="n">
-        <v>19.39</v>
+        <v>3761.41</v>
       </c>
       <c r="F59" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" s="3" t="n">
+        <v>194</v>
+      </c>
+      <c r="H59" s="5" t="n">
         <v>3761.41</v>
       </c>
     </row>
@@ -1790,14 +2156,17 @@
       <c r="C60" s="7" t="n">
         <v>33295</v>
       </c>
-      <c r="F60" s="8" t="n">
+      <c r="E60" s="8" t="n">
         <v>814657.29</v>
       </c>
+      <c r="H60" s="9" t="n">
+        <v>605097.02</v>
+      </c>
     </row>
     <row r="62">
-      <c r="B62" s="9" t="inlineStr">
-        <is>
-          <t>Период 25.06.2026–01.11.2026 = 129 дн. Хранение = дневная ставка за ед. × 129 дн × остаток без ЧЗ.</t>
+      <c r="B62" s="10" t="inlineStr">
+        <is>
+          <t>Период 25.06.2026–01.11.2026 = 129 дн. Колонка 'без продаж' = ставка×129дн×остаток. Прогноз с продажами: остаток списывается ежедневно на тек. темп продаж (продано за 8 дн ÷ 8); хранение начисляется на остаток каждый день, пока он не закончится. Темп продаж фиксированный по текущим данным.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Use funnel buyout rate (100d) for storage sales forecast
Темп продаж берётся из sales_funnel (выкупы за 01.03–09.06, 100 дн)
вместо 8-дневного окна. Хранение до ноября с учётом продаж: 623 063 руб.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RrW5WcYKgjMut1vasTMe2Q
</commit_message>
<xml_diff>
--- a/outputs/Хранение_до_ноября_без_ЧЗ.xlsx
+++ b/outputs/Хранение_до_ноября_без_ЧЗ.xlsx
@@ -472,11 +472,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
   </cols>
@@ -509,7 +509,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Продажи в день, шт (тек. темп)</t>
+          <t>Выкуп/день, шт (100 дн)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -542,13 +542,13 @@
         <v>11561.91</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>1</v>
+        <v>1.46</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>427</v>
+        <v>368</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>10231.04</v>
+        <v>9618.84</v>
       </c>
     </row>
     <row r="3">
@@ -570,13 +570,13 @@
         <v>1502.01</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.12</v>
+        <v>0.77</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>57</v>
+        <v>0</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>1337.41</v>
+        <v>557.76</v>
       </c>
     </row>
     <row r="4">
@@ -598,13 +598,13 @@
         <v>6688.65</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>1.25</v>
+        <v>1.35</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>2618.43</v>
+        <v>2426.46</v>
       </c>
     </row>
     <row r="5">
@@ -626,13 +626,13 @@
         <v>5216.14</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.75</v>
+        <v>1.11</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>3477.43</v>
+        <v>2642.84</v>
       </c>
     </row>
     <row r="6">
@@ -654,13 +654,13 @@
         <v>11266.86</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>1.38</v>
+        <v>1.94</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>373</v>
+        <v>300</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>9464.16</v>
+        <v>8723.42</v>
       </c>
     </row>
     <row r="7">
@@ -682,13 +682,13 @@
         <v>75117.47</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>2.88</v>
+        <v>3.54</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>239</v>
+        <v>153</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>52459.09</v>
+        <v>47218.11</v>
       </c>
     </row>
     <row r="8">
@@ -710,13 +710,13 @@
         <v>3563.11</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>2.38</v>
+        <v>2.9</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>1095.43</v>
+        <v>899.61</v>
       </c>
     </row>
     <row r="9">
@@ -738,13 +738,13 @@
         <v>2132.37</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>7</v>
+        <v>4.22</v>
       </c>
       <c r="G9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>126.45</v>
+        <v>204.19</v>
       </c>
     </row>
     <row r="10">
@@ -766,13 +766,13 @@
         <v>10512.57</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.5</v>
+        <v>0.86</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>432</v>
+        <v>385</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>9834.34</v>
+        <v>9346.01</v>
       </c>
     </row>
     <row r="11">
@@ -794,13 +794,13 @@
         <v>3956.69</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>3.62</v>
+        <v>3.5</v>
       </c>
       <c r="G11" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>776.92</v>
+        <v>804.12</v>
       </c>
     </row>
     <row r="12">
@@ -822,13 +822,13 @@
         <v>954.6</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0</v>
+        <v>0.11</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>954.6</v>
+        <v>820.1900000000001</v>
       </c>
     </row>
     <row r="13">
@@ -850,13 +850,13 @@
         <v>7329.97</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>345</v>
+        <v>326</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>7329.97</v>
+        <v>7126.01</v>
       </c>
     </row>
     <row r="14">
@@ -878,13 +878,13 @@
         <v>22082.99</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>4</v>
+        <v>4.16</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>592</v>
+        <v>571</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>16980.79</v>
+        <v>16776.7</v>
       </c>
     </row>
     <row r="15">
@@ -906,13 +906,13 @@
         <v>43960.94</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>23.75</v>
+        <v>2.77</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>0</v>
+        <v>2158</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>18214.08</v>
+        <v>40862.18</v>
       </c>
     </row>
     <row r="16">
@@ -934,13 +934,13 @@
         <v>48013.16</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>4.62</v>
+        <v>2.64</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>2160</v>
+        <v>2416</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>42858.31</v>
+        <v>45070.72</v>
       </c>
     </row>
     <row r="17">
@@ -962,7 +962,7 @@
         <v>0</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>2.88</v>
+        <v>0.76</v>
       </c>
       <c r="G17" s="3" t="n">
         <v>0</v>
@@ -990,13 +990,13 @@
         <v>8015.75</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>3.38</v>
+        <v>2.38</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>76</v>
+        <v>204</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>4627.49</v>
+        <v>5626.4</v>
       </c>
     </row>
     <row r="19">
@@ -1018,13 +1018,13 @@
         <v>1670.76</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>1.5</v>
+        <v>0.96</v>
       </c>
       <c r="G19" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>377.78</v>
+        <v>586.62</v>
       </c>
     </row>
     <row r="20">
@@ -1046,13 +1046,13 @@
         <v>29541.68</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>4.12</v>
+        <v>2.64</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>879</v>
+        <v>1070</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>24014.39</v>
+        <v>26004.22</v>
       </c>
     </row>
     <row r="21">
@@ -1074,13 +1074,13 @@
         <v>10115.44</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>9.619999999999999</v>
+        <v>2.97</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>0</v>
+        <v>194</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>2389.63</v>
+        <v>6783.13</v>
       </c>
     </row>
     <row r="22">
@@ -1102,13 +1102,13 @@
         <v>4626.07</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>5</v>
+        <v>3.6</v>
       </c>
       <c r="G22" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>860.66</v>
+        <v>1188.45</v>
       </c>
     </row>
     <row r="23">
@@ -1130,13 +1130,13 @@
         <v>639.71</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>4.5</v>
+        <v>2.94</v>
       </c>
       <c r="G23" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>19.09</v>
+        <v>27.82</v>
       </c>
     </row>
     <row r="24">
@@ -1158,13 +1158,13 @@
         <v>15404.87</v>
       </c>
       <c r="F24" s="5" t="n">
-        <v>4.12</v>
+        <v>2.2</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>262</v>
+        <v>510</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>10282.85</v>
+        <v>12673.13</v>
       </c>
     </row>
     <row r="25">
@@ -1186,13 +1186,13 @@
         <v>16629.24</v>
       </c>
       <c r="F25" s="5" t="n">
-        <v>2.25</v>
+        <v>1.96</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>574</v>
+        <v>611</v>
       </c>
       <c r="H25" s="5" t="n">
-        <v>13857.7</v>
+        <v>14214.92</v>
       </c>
     </row>
     <row r="26">
@@ -1214,13 +1214,13 @@
         <v>18261.11</v>
       </c>
       <c r="F26" s="5" t="n">
-        <v>1</v>
+        <v>1.39</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>806</v>
+        <v>756</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>17011.15</v>
+        <v>16523.67</v>
       </c>
     </row>
     <row r="27">
@@ -1242,13 +1242,13 @@
         <v>7857.51</v>
       </c>
       <c r="F27" s="5" t="n">
-        <v>13.12</v>
+        <v>27.54</v>
       </c>
       <c r="G27" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H27" s="5" t="n">
-        <v>896.23</v>
+        <v>443.5</v>
       </c>
     </row>
     <row r="28">
@@ -1270,13 +1270,13 @@
         <v>8651.059999999999</v>
       </c>
       <c r="F28" s="5" t="n">
-        <v>2</v>
+        <v>2.82</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>467</v>
+        <v>361</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>7123.7</v>
+        <v>6497.48</v>
       </c>
     </row>
     <row r="29">
@@ -1298,13 +1298,13 @@
         <v>6327.6</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>2.12</v>
+        <v>2.09</v>
       </c>
       <c r="G29" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H29" s="5" t="n">
-        <v>3071.51</v>
+        <v>3122.54</v>
       </c>
     </row>
     <row r="30">
@@ -1326,13 +1326,13 @@
         <v>127609.84</v>
       </c>
       <c r="F30" s="5" t="n">
-        <v>14.38</v>
+        <v>14.06</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>1414</v>
+        <v>1454</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>91685.41</v>
+        <v>92472.62</v>
       </c>
     </row>
     <row r="31">
@@ -1354,13 +1354,13 @@
         <v>107923.73</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>9.880000000000001</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>2907</v>
+        <v>2918</v>
       </c>
       <c r="H31" s="5" t="n">
-        <v>91609.98</v>
+        <v>91750.39999999999</v>
       </c>
     </row>
     <row r="32">
@@ -1382,13 +1382,13 @@
         <v>11605.36</v>
       </c>
       <c r="F32" s="5" t="n">
-        <v>5.5</v>
+        <v>5.3</v>
       </c>
       <c r="G32" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>4911.28</v>
+        <v>5094.93</v>
       </c>
     </row>
     <row r="33">
@@ -1410,13 +1410,13 @@
         <v>9613.139999999999</v>
       </c>
       <c r="F33" s="5" t="n">
-        <v>1.12</v>
+        <v>1.74</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>370</v>
+        <v>291</v>
       </c>
       <c r="H33" s="5" t="n">
-        <v>8269.17</v>
+        <v>7534.47</v>
       </c>
     </row>
     <row r="34">
@@ -1438,13 +1438,13 @@
         <v>2135.87</v>
       </c>
       <c r="F34" s="5" t="n">
-        <v>1.5</v>
+        <v>1.79</v>
       </c>
       <c r="G34" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>609.88</v>
+        <v>512.4</v>
       </c>
     </row>
     <row r="35">
@@ -1466,13 +1466,13 @@
         <v>753.84</v>
       </c>
       <c r="F35" s="5" t="n">
-        <v>0.25</v>
+        <v>0.44</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="H35" s="5" t="n">
-        <v>473.34</v>
+        <v>288.47</v>
       </c>
     </row>
     <row r="36">
@@ -1494,13 +1494,13 @@
         <v>2661.73</v>
       </c>
       <c r="F36" s="5" t="n">
-        <v>1</v>
+        <v>1.12</v>
       </c>
       <c r="G36" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>1330.87</v>
+        <v>1189.4</v>
       </c>
     </row>
     <row r="37">
@@ -1522,13 +1522,13 @@
         <v>32719.84</v>
       </c>
       <c r="F37" s="5" t="n">
-        <v>0.88</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>1270</v>
+        <v>1294</v>
       </c>
       <c r="H37" s="5" t="n">
-        <v>31394.96</v>
+        <v>31675.08</v>
       </c>
     </row>
     <row r="38">
@@ -1550,13 +1550,13 @@
         <v>25418.44</v>
       </c>
       <c r="F38" s="5" t="n">
-        <v>1.62</v>
+        <v>3.34</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>832</v>
+        <v>611</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>22881.48</v>
+        <v>20204</v>
       </c>
     </row>
     <row r="39">
@@ -1578,13 +1578,13 @@
         <v>19862.65</v>
       </c>
       <c r="F39" s="5" t="n">
-        <v>1.75</v>
+        <v>5.9</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>609</v>
+        <v>74</v>
       </c>
       <c r="H39" s="5" t="n">
-        <v>17198.43</v>
+        <v>10880.45</v>
       </c>
     </row>
     <row r="40">
@@ -1606,13 +1606,13 @@
         <v>8311.209999999999</v>
       </c>
       <c r="F40" s="5" t="n">
-        <v>0.12</v>
+        <v>0.74</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>404</v>
+        <v>325</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>8152.9</v>
+        <v>7374.02</v>
       </c>
     </row>
     <row r="41">
@@ -1634,13 +1634,13 @@
         <v>12284.26</v>
       </c>
       <c r="F41" s="5" t="n">
-        <v>6.75</v>
+        <v>2.71</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>0</v>
+        <v>284</v>
       </c>
       <c r="H41" s="5" t="n">
-        <v>4519.78</v>
+        <v>8923.719999999999</v>
       </c>
     </row>
     <row r="42">
@@ -1662,13 +1662,13 @@
         <v>5136.44</v>
       </c>
       <c r="F42" s="5" t="n">
-        <v>0.25</v>
+        <v>0.72</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>87</v>
+        <v>26</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>4445.83</v>
+        <v>3147.48</v>
       </c>
     </row>
     <row r="43">
@@ -1690,13 +1690,13 @@
         <v>1805.55</v>
       </c>
       <c r="F43" s="5" t="n">
-        <v>0.88</v>
+        <v>0.65</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="H43" s="5" t="n">
-        <v>846.79</v>
+        <v>1090.21</v>
       </c>
     </row>
     <row r="44">
@@ -1718,13 +1718,13 @@
         <v>6010.11</v>
       </c>
       <c r="F44" s="5" t="n">
-        <v>1.25</v>
+        <v>2.08</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>139</v>
+        <v>32</v>
       </c>
       <c r="H44" s="5" t="n">
-        <v>4407.41</v>
+        <v>3343.22</v>
       </c>
     </row>
     <row r="45">
@@ -1746,13 +1746,13 @@
         <v>4531.38</v>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0.5</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>206</v>
+        <v>181</v>
       </c>
       <c r="H45" s="5" t="n">
-        <v>3994.33</v>
+        <v>3790.25</v>
       </c>
     </row>
     <row r="46">
@@ -1774,13 +1774,13 @@
         <v>11029.44</v>
       </c>
       <c r="F46" s="5" t="n">
-        <v>1.38</v>
+        <v>1.09</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>380</v>
+        <v>416</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>9286.9</v>
+        <v>9648.08</v>
       </c>
     </row>
     <row r="47">
@@ -1802,13 +1802,13 @@
         <v>4472.56</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>1.75</v>
+        <v>1.14</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="H47" s="5" t="n">
-        <v>2097.6</v>
+        <v>2918.66</v>
       </c>
     </row>
     <row r="48">
@@ -1830,13 +1830,13 @@
         <v>1532.52</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>1</v>
+        <v>1.07</v>
       </c>
       <c r="G48" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>451.44</v>
+        <v>422.3</v>
       </c>
     </row>
     <row r="49">
@@ -1858,13 +1858,13 @@
         <v>1699.19</v>
       </c>
       <c r="F49" s="5" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="H49" s="5" t="n">
-        <v>1393.72</v>
+        <v>1088.24</v>
       </c>
     </row>
     <row r="50">
@@ -1886,13 +1886,13 @@
         <v>1551.44</v>
       </c>
       <c r="F50" s="5" t="n">
-        <v>0.25</v>
+        <v>0.15</v>
       </c>
       <c r="G50" s="3" t="n">
-        <v>51</v>
+        <v>64</v>
       </c>
       <c r="H50" s="5" t="n">
-        <v>1252.37</v>
+        <v>1372</v>
       </c>
     </row>
     <row r="51">
@@ -1914,13 +1914,13 @@
         <v>9388.450000000001</v>
       </c>
       <c r="F51" s="5" t="n">
-        <v>0.12</v>
+        <v>0.05</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>511</v>
+        <v>521</v>
       </c>
       <c r="H51" s="5" t="n">
-        <v>9245.93</v>
+        <v>9331.440000000001</v>
       </c>
     </row>
     <row r="52">
@@ -1942,13 +1942,13 @@
         <v>1185.57</v>
       </c>
       <c r="F52" s="5" t="n">
-        <v>0.25</v>
+        <v>0.28</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="H52" s="5" t="n">
-        <v>840.6799999999999</v>
+        <v>799.29</v>
       </c>
     </row>
     <row r="53">
@@ -1970,13 +1970,13 @@
         <v>2435.52</v>
       </c>
       <c r="F53" s="5" t="n">
-        <v>0.75</v>
+        <v>0.63</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="H53" s="5" t="n">
-        <v>1444.8</v>
+        <v>1603.32</v>
       </c>
     </row>
     <row r="54">
@@ -1998,13 +1998,13 @@
         <v>635.71</v>
       </c>
       <c r="F54" s="5" t="n">
-        <v>0.12</v>
+        <v>0.21</v>
       </c>
       <c r="G54" s="3" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="H54" s="5" t="n">
-        <v>476.78</v>
+        <v>368.71</v>
       </c>
     </row>
     <row r="55">
@@ -2026,13 +2026,13 @@
         <v>2028.03</v>
       </c>
       <c r="F55" s="5" t="n">
-        <v>0.12</v>
+        <v>0.17</v>
       </c>
       <c r="G55" s="3" t="n">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="H55" s="5" t="n">
-        <v>1864.15</v>
+        <v>1805.16</v>
       </c>
     </row>
     <row r="56">
@@ -2054,13 +2054,13 @@
         <v>10644.4</v>
       </c>
       <c r="F56" s="5" t="n">
-        <v>0.25</v>
+        <v>0.19</v>
       </c>
       <c r="G56" s="3" t="n">
-        <v>469</v>
+        <v>476</v>
       </c>
       <c r="H56" s="5" t="n">
-        <v>10304.46</v>
+        <v>10386.04</v>
       </c>
     </row>
     <row r="57">
@@ -2082,13 +2082,13 @@
         <v>1719.67</v>
       </c>
       <c r="F57" s="5" t="n">
-        <v>0.5</v>
+        <v>0.34</v>
       </c>
       <c r="G57" s="3" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="H57" s="5" t="n">
-        <v>1064.56</v>
+        <v>1274.2</v>
       </c>
     </row>
     <row r="58">
@@ -2110,13 +2110,13 @@
         <v>2589.75</v>
       </c>
       <c r="F58" s="5" t="n">
-        <v>0</v>
+        <v>0.19</v>
       </c>
       <c r="G58" s="3" t="n">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="H58" s="5" t="n">
-        <v>2589.75</v>
+        <v>2335.79</v>
       </c>
     </row>
     <row r="59">
@@ -2138,13 +2138,13 @@
         <v>3761.41</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="G59" s="3" t="n">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="H59" s="5" t="n">
-        <v>3761.41</v>
+        <v>3649.73</v>
       </c>
     </row>
     <row r="60">
@@ -2160,13 +2160,13 @@
         <v>814657.29</v>
       </c>
       <c r="H60" s="9" t="n">
-        <v>605097.02</v>
+        <v>623063.12</v>
       </c>
     </row>
     <row r="62">
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>Период 25.06.2026–01.11.2026 = 129 дн. Колонка 'без продаж' = ставка×129дн×остаток. Прогноз с продажами: остаток списывается ежедневно на тек. темп продаж (продано за 8 дн ÷ 8); хранение начисляется на остаток каждый день, пока он не закончится. Темп продаж фиксированный по текущим данным.</t>
+          <t>Период хранения 25.06.2026–01.11.2026 = 129 дн. Темп продаж = выкупы из отчёта 'Воронка продаж' за 01.03–09.06.2026 (100 дн) ÷ 100. Прогноз: остаток списывается ежедневно на этот темп, хранение начисляется на остаток до распродажи или до 01.11. Темп фиксированный.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add seasonality-adjusted storage forecast until November
Сезонные коэффициенты по месяцам (якоря: зима/весна из воронки,
лето-осень — оценка по категории), вынесены на лист 'Сезонность'.
Хранение до ноября с сезонностью: 630 089 руб.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RrW5WcYKgjMut1vasTMe2Q
</commit_message>
<xml_diff>
--- a/outputs/Хранение_до_ноября_без_ЧЗ.xlsx
+++ b/outputs/Хранение_до_ноября_без_ЧЗ.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Хранение до ноября (без ЧЗ)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Сезонность" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -40,7 +41,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -55,6 +56,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -89,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -102,7 +108,9 @@
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -468,17 +476,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -504,22 +513,27 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Хранение до ноября всего (без продаж), руб</t>
+          <t>Хранение до ноября (без продаж), руб</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Выкуп/день, шт (100 дн)</t>
+          <t>Выкуп/день базовый, шт</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Прогноз остатка к 01.11, шт</t>
+          <t>Прогноз остатка к 01.11 (с сезонностью), шт</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Хранение до ноября с учётом продаж, руб</t>
+          <t>Хранение до ноября без сезонности, руб</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Хранение до ноября С СЕЗОННОСТЬЮ, руб</t>
         </is>
       </c>
     </row>
@@ -545,10 +559,13 @@
         <v>1.46</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="H2" s="5" t="n">
         <v>9618.84</v>
+      </c>
+      <c r="I2" s="5" t="n">
+        <v>9696.459999999999</v>
       </c>
     </row>
     <row r="3">
@@ -578,6 +595,9 @@
       <c r="H3" s="5" t="n">
         <v>557.76</v>
       </c>
+      <c r="I3" s="5" t="n">
+        <v>591.54</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -606,6 +626,9 @@
       <c r="H4" s="5" t="n">
         <v>2426.46</v>
       </c>
+      <c r="I4" s="5" t="n">
+        <v>2576.08</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -634,6 +657,9 @@
       <c r="H5" s="5" t="n">
         <v>2642.84</v>
       </c>
+      <c r="I5" s="5" t="n">
+        <v>2745.64</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -657,10 +683,13 @@
         <v>1.94</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H6" s="5" t="n">
         <v>8723.42</v>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>8825.02</v>
       </c>
     </row>
     <row r="7">
@@ -685,10 +714,13 @@
         <v>3.54</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="H7" s="5" t="n">
         <v>47218.11</v>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>48332.56</v>
       </c>
     </row>
     <row r="8">
@@ -718,6 +750,9 @@
       <c r="H8" s="5" t="n">
         <v>899.61</v>
       </c>
+      <c r="I8" s="5" t="n">
+        <v>962.85</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -746,6 +781,9 @@
       <c r="H9" s="5" t="n">
         <v>204.19</v>
       </c>
+      <c r="I9" s="5" t="n">
+        <v>213.67</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -774,6 +812,9 @@
       <c r="H10" s="5" t="n">
         <v>9346.01</v>
       </c>
+      <c r="I10" s="5" t="n">
+        <v>9392.610000000001</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -802,6 +843,9 @@
       <c r="H11" s="5" t="n">
         <v>804.12</v>
       </c>
+      <c r="I11" s="5" t="n">
+        <v>857.62</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -830,6 +874,9 @@
       <c r="H12" s="5" t="n">
         <v>820.1900000000001</v>
       </c>
+      <c r="I12" s="5" t="n">
+        <v>825.5599999999999</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -858,6 +905,9 @@
       <c r="H13" s="5" t="n">
         <v>7126.01</v>
       </c>
+      <c r="I13" s="5" t="n">
+        <v>7134.16</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -881,10 +931,13 @@
         <v>4.16</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="H14" s="5" t="n">
         <v>16776.7</v>
+      </c>
+      <c r="I14" s="5" t="n">
+        <v>16988.66</v>
       </c>
     </row>
     <row r="15">
@@ -909,10 +962,13 @@
         <v>2.77</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>2158</v>
+        <v>2157</v>
       </c>
       <c r="H15" s="5" t="n">
         <v>40862.18</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>40985.96</v>
       </c>
     </row>
     <row r="16">
@@ -942,6 +998,9 @@
       <c r="H16" s="5" t="n">
         <v>45070.72</v>
       </c>
+      <c r="I16" s="5" t="n">
+        <v>45188.25</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -970,6 +1029,9 @@
       <c r="H17" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="I17" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -993,10 +1055,13 @@
         <v>2.38</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="H18" s="5" t="n">
         <v>5626.4</v>
+      </c>
+      <c r="I18" s="5" t="n">
+        <v>5721.84</v>
       </c>
     </row>
     <row r="19">
@@ -1026,6 +1091,9 @@
       <c r="H19" s="5" t="n">
         <v>586.62</v>
       </c>
+      <c r="I19" s="5" t="n">
+        <v>623.6799999999999</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1054,6 +1122,9 @@
       <c r="H20" s="5" t="n">
         <v>26004.22</v>
       </c>
+      <c r="I20" s="5" t="n">
+        <v>26145.52</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1077,10 +1148,13 @@
         <v>2.97</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="H21" s="5" t="n">
         <v>6783.13</v>
+      </c>
+      <c r="I21" s="5" t="n">
+        <v>6916.24</v>
       </c>
     </row>
     <row r="22">
@@ -1110,6 +1184,9 @@
       <c r="H22" s="5" t="n">
         <v>1188.45</v>
       </c>
+      <c r="I22" s="5" t="n">
+        <v>1272.17</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1138,6 +1215,9 @@
       <c r="H23" s="5" t="n">
         <v>27.82</v>
       </c>
+      <c r="I23" s="5" t="n">
+        <v>28.21</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1166,6 +1246,9 @@
       <c r="H24" s="5" t="n">
         <v>12673.13</v>
       </c>
+      <c r="I24" s="5" t="n">
+        <v>12782.25</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1194,6 +1277,9 @@
       <c r="H25" s="5" t="n">
         <v>14214.92</v>
       </c>
+      <c r="I25" s="5" t="n">
+        <v>14311.36</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1217,10 +1303,13 @@
         <v>1.39</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="H26" s="5" t="n">
         <v>16523.67</v>
+      </c>
+      <c r="I26" s="5" t="n">
+        <v>16593.07</v>
       </c>
     </row>
     <row r="27">
@@ -1250,6 +1339,9 @@
       <c r="H27" s="5" t="n">
         <v>443.5</v>
       </c>
+      <c r="I27" s="5" t="n">
+        <v>454.4</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1273,10 +1365,13 @@
         <v>2.82</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="H28" s="5" t="n">
         <v>6497.48</v>
+      </c>
+      <c r="I28" s="5" t="n">
+        <v>6583.51</v>
       </c>
     </row>
     <row r="29">
@@ -1306,6 +1401,9 @@
       <c r="H29" s="5" t="n">
         <v>3122.54</v>
       </c>
+      <c r="I29" s="5" t="n">
+        <v>3250.66</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -1329,10 +1427,13 @@
         <v>14.06</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>1454</v>
+        <v>1451</v>
       </c>
       <c r="H30" s="5" t="n">
         <v>92472.62</v>
+      </c>
+      <c r="I30" s="5" t="n">
+        <v>93876.2</v>
       </c>
     </row>
     <row r="31">
@@ -1357,10 +1458,13 @@
         <v>9.789999999999999</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>2918</v>
+        <v>2916</v>
       </c>
       <c r="H31" s="5" t="n">
         <v>91750.39999999999</v>
+      </c>
+      <c r="I31" s="5" t="n">
+        <v>92396.46000000001</v>
       </c>
     </row>
     <row r="32">
@@ -1390,6 +1494,9 @@
       <c r="H32" s="5" t="n">
         <v>5094.93</v>
       </c>
+      <c r="I32" s="5" t="n">
+        <v>5350.2</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -1413,10 +1520,13 @@
         <v>1.74</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H33" s="5" t="n">
         <v>7534.47</v>
+      </c>
+      <c r="I33" s="5" t="n">
+        <v>7617.5</v>
       </c>
     </row>
     <row r="34">
@@ -1446,6 +1556,9 @@
       <c r="H34" s="5" t="n">
         <v>512.4</v>
       </c>
+      <c r="I34" s="5" t="n">
+        <v>548.04</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -1474,6 +1587,9 @@
       <c r="H35" s="5" t="n">
         <v>288.47</v>
       </c>
+      <c r="I35" s="5" t="n">
+        <v>305.49</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -1502,6 +1618,9 @@
       <c r="H36" s="5" t="n">
         <v>1189.4</v>
       </c>
+      <c r="I36" s="5" t="n">
+        <v>1247.45</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -1530,6 +1649,9 @@
       <c r="H37" s="5" t="n">
         <v>31675.08</v>
       </c>
+      <c r="I37" s="5" t="n">
+        <v>31716.81</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -1553,10 +1675,13 @@
         <v>3.34</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="H38" s="5" t="n">
         <v>20204</v>
+      </c>
+      <c r="I38" s="5" t="n">
+        <v>20412.3</v>
       </c>
     </row>
     <row r="39">
@@ -1581,10 +1706,13 @@
         <v>5.9</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H39" s="5" t="n">
         <v>10880.45</v>
+      </c>
+      <c r="I39" s="5" t="n">
+        <v>11239.25</v>
       </c>
     </row>
     <row r="40">
@@ -1609,10 +1737,13 @@
         <v>0.74</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="H40" s="5" t="n">
         <v>7374.02</v>
+      </c>
+      <c r="I40" s="5" t="n">
+        <v>7411.46</v>
       </c>
     </row>
     <row r="41">
@@ -1642,6 +1773,9 @@
       <c r="H41" s="5" t="n">
         <v>8923.719999999999</v>
       </c>
+      <c r="I41" s="5" t="n">
+        <v>9057.959999999999</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -1670,6 +1804,9 @@
       <c r="H42" s="5" t="n">
         <v>3147.48</v>
       </c>
+      <c r="I42" s="5" t="n">
+        <v>3226.93</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -1698,6 +1835,9 @@
       <c r="H43" s="5" t="n">
         <v>1090.21</v>
       </c>
+      <c r="I43" s="5" t="n">
+        <v>1118.78</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -1721,10 +1861,13 @@
         <v>2.08</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H44" s="5" t="n">
         <v>3343.22</v>
+      </c>
+      <c r="I44" s="5" t="n">
+        <v>3449.75</v>
       </c>
     </row>
     <row r="45">
@@ -1754,6 +1897,9 @@
       <c r="H45" s="5" t="n">
         <v>3790.25</v>
       </c>
+      <c r="I45" s="5" t="n">
+        <v>3819.86</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -1782,6 +1928,9 @@
       <c r="H46" s="5" t="n">
         <v>9648.08</v>
       </c>
+      <c r="I46" s="5" t="n">
+        <v>9703.26</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -1810,6 +1959,9 @@
       <c r="H47" s="5" t="n">
         <v>2918.66</v>
       </c>
+      <c r="I47" s="5" t="n">
+        <v>2980.74</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -1838,6 +1990,9 @@
       <c r="H48" s="5" t="n">
         <v>422.3</v>
       </c>
+      <c r="I48" s="5" t="n">
+        <v>452.02</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -1866,6 +2021,9 @@
       <c r="H49" s="5" t="n">
         <v>1088.24</v>
       </c>
+      <c r="I49" s="5" t="n">
+        <v>1112.65</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -1894,6 +2052,9 @@
       <c r="H50" s="5" t="n">
         <v>1372</v>
       </c>
+      <c r="I50" s="5" t="n">
+        <v>1379.17</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -1922,6 +2083,9 @@
       <c r="H51" s="5" t="n">
         <v>9331.440000000001</v>
       </c>
+      <c r="I51" s="5" t="n">
+        <v>9333.719999999999</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -1950,6 +2114,9 @@
       <c r="H52" s="5" t="n">
         <v>799.29</v>
       </c>
+      <c r="I52" s="5" t="n">
+        <v>814.72</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -1978,6 +2145,9 @@
       <c r="H53" s="5" t="n">
         <v>1603.32</v>
       </c>
+      <c r="I53" s="5" t="n">
+        <v>1636.56</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -2006,6 +2176,9 @@
       <c r="H54" s="5" t="n">
         <v>368.71</v>
       </c>
+      <c r="I54" s="5" t="n">
+        <v>379.38</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -2034,6 +2207,9 @@
       <c r="H55" s="5" t="n">
         <v>1805.16</v>
       </c>
+      <c r="I55" s="5" t="n">
+        <v>1814.06</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -2062,6 +2238,9 @@
       <c r="H56" s="5" t="n">
         <v>10386.04</v>
       </c>
+      <c r="I56" s="5" t="n">
+        <v>10396.36</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -2090,6 +2269,9 @@
       <c r="H57" s="5" t="n">
         <v>1274.2</v>
       </c>
+      <c r="I57" s="5" t="n">
+        <v>1291.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -2118,6 +2300,9 @@
       <c r="H58" s="5" t="n">
         <v>2335.79</v>
       </c>
+      <c r="I58" s="5" t="n">
+        <v>2345.93</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -2146,6 +2331,9 @@
       <c r="H59" s="5" t="n">
         <v>3649.73</v>
       </c>
+      <c r="I59" s="5" t="n">
+        <v>3654.19</v>
+      </c>
     </row>
     <row r="60">
       <c r="B60" s="6" t="inlineStr">
@@ -2157,18 +2345,182 @@
         <v>33295</v>
       </c>
       <c r="E60" s="8" t="n">
-        <v>814657.29</v>
+        <v>814657.33</v>
       </c>
       <c r="H60" s="9" t="n">
         <v>623063.12</v>
       </c>
+      <c r="I60" s="10" t="n">
+        <v>630088.73</v>
+      </c>
     </row>
     <row r="62">
-      <c r="B62" s="10" t="inlineStr">
-        <is>
-          <t>Период хранения 25.06.2026–01.11.2026 = 129 дн. Темп продаж = выкупы из отчёта 'Воронка продаж' за 01.03–09.06.2026 (100 дн) ÷ 100. Прогноз: остаток списывается ежедневно на этот темп, хранение начисляется на остаток до распродажи или до 01.11. Темп фиксированный.</t>
-        </is>
-      </c>
+      <c r="B62" s="11" t="inlineStr">
+        <is>
+          <t>Период 25.06–01.11.2026 = 129 дн. Базовый темп = выкупы за весну (01.03–09.06) ÷ 100. Сезонность: дневной темп = базовый × коэф месяца (лист 'Сезонность'). Остаток списывается ежедневно, хранение на остаток до распродажи или 01.11. Лето/осень оценочно (прямых данных по этим месяцам нет): зима/весна — из выгрузок, лето-спад/осень-рост — по сезонности категории.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Месяц</t>
+        </is>
+      </c>
+      <c r="B1" s="12" t="inlineStr">
+        <is>
+          <t>Сезонный коэффициент (база весна=1.00)</t>
+        </is>
+      </c>
+      <c r="C1" s="12" t="inlineStr">
+        <is>
+          <t>Комментарий</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Июнь</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>конец весеннего окна (данные)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Июль</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>лето, спад по уходу</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Август</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>лето, спад по уходу</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Сентябрь</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>осень, восстановление</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Октябрь</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>предсезонный рост</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Ноябрь</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ноябрь, высокий сезон</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Якоря из данных воронки:</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Зима 20.11–28.02 (выкупы)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>124.6 шт/день → коэф 0.87</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Весна 01.03–09.06 (выкупы)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>143.6 шт/день → коэф 1.00 (база)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>